<commit_message>
feat: bugfix JWT/CORS and finish sprint 3
</commit_message>
<xml_diff>
--- a/docs/Producto_Backlog_V1.0.xlsx
+++ b/docs/Producto_Backlog_V1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jhoan\Documents\Programacion\posSYSTEM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF7787D6-8697-4C1E-A85F-903D83E69CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39E53EF1-BA16-4ACC-9414-6F460BDAECF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="134">
   <si>
     <t>Columna</t>
   </si>
@@ -429,6 +429,12 @@
   </si>
   <si>
     <t>Identificar mejores clientes.</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -570,7 +576,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -582,6 +588,20 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -591,13 +611,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -606,18 +622,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -923,7 +927,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:I76"/>
+  <dimension ref="B1:G76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="1.44140625" style="2" customWidth="1"/>
@@ -949,7 +953,7 @@
       <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="7" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="6" t="s">
@@ -966,14 +970,16 @@
       </c>
     </row>
     <row r="5" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="7" t="s">
+      <c r="D5" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E5" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -982,56 +988,62 @@
       <c r="G5" s="5"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="8"/>
+      <c r="D6" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E6" s="14"/>
       <c r="F6" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G6" s="5"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="8"/>
+      <c r="D7" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E7" s="14"/>
       <c r="F7" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G7" s="5"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="9"/>
+      <c r="D8" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8" s="15"/>
       <c r="F8" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G8" s="5"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="8" t="s">
         <v>42</v>
       </c>
       <c r="D9" s="5"/>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="13" t="s">
         <v>41</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -1040,168 +1052,168 @@
       <c r="G9" s="5"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="8" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="5"/>
-      <c r="E10" s="8"/>
+      <c r="E10" s="14"/>
       <c r="F10" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G10" s="5"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="8" t="s">
         <v>44</v>
       </c>
       <c r="D11" s="5"/>
-      <c r="E11" s="8"/>
+      <c r="E11" s="14"/>
       <c r="F11" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G11" s="5"/>
     </row>
     <row r="12" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="8" t="s">
         <v>45</v>
       </c>
       <c r="D12" s="5"/>
-      <c r="E12" s="8"/>
+      <c r="E12" s="14"/>
       <c r="F12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G12" s="5"/>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D13" s="5"/>
-      <c r="E13" s="8"/>
+      <c r="E13" s="14"/>
       <c r="F13" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="8" t="s">
         <v>47</v>
       </c>
       <c r="D14" s="5"/>
-      <c r="E14" s="8"/>
+      <c r="E14" s="14"/>
       <c r="F14" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G14" s="5"/>
     </row>
     <row r="15" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="8" t="s">
         <v>48</v>
       </c>
       <c r="D15" s="5"/>
-      <c r="E15" s="8"/>
+      <c r="E15" s="14"/>
       <c r="F15" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G15" s="5"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="8" t="s">
         <v>50</v>
       </c>
       <c r="D16" s="5"/>
-      <c r="E16" s="8"/>
+      <c r="E16" s="14"/>
       <c r="F16" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G16" s="5"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="8" t="s">
         <v>51</v>
       </c>
       <c r="D17" s="5"/>
-      <c r="E17" s="8"/>
+      <c r="E17" s="14"/>
       <c r="F17" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G17" s="5"/>
     </row>
     <row r="18" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="8" t="s">
         <v>88</v>
       </c>
       <c r="D18" s="5"/>
-      <c r="E18" s="8"/>
+      <c r="E18" s="14"/>
       <c r="F18" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G18" s="5"/>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="9" t="s">
         <v>89</v>
       </c>
       <c r="D19" s="5"/>
-      <c r="E19" s="8"/>
+      <c r="E19" s="14"/>
       <c r="F19" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G19" s="5"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="9" t="s">
         <v>90</v>
       </c>
       <c r="D20" s="5"/>
-      <c r="E20" s="9"/>
+      <c r="E20" s="15"/>
       <c r="F20" s="5" t="s">
         <v>91</v>
       </c>
       <c r="G20" s="5"/>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="9" t="s">
         <v>93</v>
       </c>
       <c r="D21" s="5"/>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="13" t="s">
         <v>92</v>
       </c>
       <c r="F21" s="5" t="s">
@@ -1210,56 +1222,56 @@
       <c r="G21" s="5"/>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="9" t="s">
         <v>94</v>
       </c>
       <c r="D22" s="5"/>
-      <c r="E22" s="8"/>
+      <c r="E22" s="14"/>
       <c r="F22" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G22" s="5"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="9" t="s">
         <v>95</v>
       </c>
       <c r="D23" s="5"/>
-      <c r="E23" s="8"/>
+      <c r="E23" s="14"/>
       <c r="F23" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G23" s="5"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="9" t="s">
         <v>96</v>
       </c>
       <c r="D24" s="5"/>
-      <c r="E24" s="9"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="5" t="s">
         <v>91</v>
       </c>
       <c r="G24" s="5"/>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="9" t="s">
         <v>98</v>
       </c>
       <c r="D25" s="5"/>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="13" t="s">
         <v>97</v>
       </c>
       <c r="F25" s="5" t="s">
@@ -1268,56 +1280,56 @@
       <c r="G25" s="5"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="9" t="s">
         <v>99</v>
       </c>
       <c r="D26" s="5"/>
-      <c r="E26" s="8"/>
+      <c r="E26" s="14"/>
       <c r="F26" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G26" s="5"/>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="9" t="s">
         <v>100</v>
       </c>
       <c r="D27" s="5"/>
-      <c r="E27" s="8"/>
+      <c r="E27" s="14"/>
       <c r="F27" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G27" s="5"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B28" s="12" t="s">
+      <c r="B28" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="9" t="s">
         <v>101</v>
       </c>
       <c r="D28" s="5"/>
-      <c r="E28" s="9"/>
+      <c r="E28" s="15"/>
       <c r="F28" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G28" s="5"/>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" s="9" t="s">
         <v>102</v>
       </c>
       <c r="D29" s="5"/>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="17" t="s">
         <v>107</v>
       </c>
       <c r="F29" s="5" t="s">
@@ -1326,70 +1338,70 @@
       <c r="G29" s="5"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="9" t="s">
         <v>103</v>
       </c>
       <c r="D30" s="5"/>
-      <c r="E30" s="14"/>
+      <c r="E30" s="18"/>
       <c r="F30" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G30" s="5"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="9" t="s">
         <v>104</v>
       </c>
       <c r="D31" s="5"/>
-      <c r="E31" s="14"/>
+      <c r="E31" s="18"/>
       <c r="F31" s="5" t="s">
         <v>23</v>
       </c>
       <c r="G31" s="5"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="9" t="s">
         <v>105</v>
       </c>
       <c r="D32" s="5"/>
-      <c r="E32" s="14"/>
+      <c r="E32" s="18"/>
       <c r="F32" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G32" s="5"/>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="C33" s="9" t="s">
         <v>106</v>
       </c>
       <c r="D33" s="5"/>
-      <c r="E33" s="15"/>
+      <c r="E33" s="19"/>
       <c r="F33" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G33" s="5"/>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C34" s="9" t="s">
         <v>109</v>
       </c>
       <c r="D34" s="5"/>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="13" t="s">
         <v>108</v>
       </c>
       <c r="F34" s="5" t="s">
@@ -1398,70 +1410,70 @@
       <c r="G34" s="5"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B35" s="12" t="s">
+      <c r="B35" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="9" t="s">
         <v>110</v>
       </c>
       <c r="D35" s="5"/>
-      <c r="E35" s="8"/>
+      <c r="E35" s="14"/>
       <c r="F35" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G35" s="5"/>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="C36" s="9" t="s">
         <v>111</v>
       </c>
       <c r="D36" s="5"/>
-      <c r="E36" s="8"/>
+      <c r="E36" s="14"/>
       <c r="F36" s="5" t="s">
         <v>91</v>
       </c>
       <c r="G36" s="5"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="9" t="s">
         <v>112</v>
       </c>
       <c r="D37" s="5"/>
-      <c r="E37" s="8"/>
+      <c r="E37" s="14"/>
       <c r="F37" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G37" s="5"/>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C38" s="12" t="s">
+      <c r="C38" s="9" t="s">
         <v>113</v>
       </c>
       <c r="D38" s="5"/>
-      <c r="E38" s="9"/>
+      <c r="E38" s="15"/>
       <c r="F38" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G38" s="5"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C39" s="12" t="s">
+      <c r="C39" s="9" t="s">
         <v>114</v>
       </c>
       <c r="D39" s="5"/>
-      <c r="E39" s="7" t="s">
+      <c r="E39" s="13" t="s">
         <v>122</v>
       </c>
       <c r="F39" s="5" t="s">
@@ -1470,98 +1482,98 @@
       <c r="G39" s="5"/>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="C40" s="9" t="s">
         <v>115</v>
       </c>
       <c r="D40" s="5"/>
-      <c r="E40" s="8"/>
+      <c r="E40" s="14"/>
       <c r="F40" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G40" s="5"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="C41" s="9" t="s">
         <v>116</v>
       </c>
       <c r="D41" s="5"/>
-      <c r="E41" s="8"/>
+      <c r="E41" s="14"/>
       <c r="F41" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G41" s="5"/>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B42" s="12" t="s">
+      <c r="B42" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="C42" s="9" t="s">
         <v>117</v>
       </c>
       <c r="D42" s="5"/>
-      <c r="E42" s="8"/>
+      <c r="E42" s="14"/>
       <c r="F42" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G42" s="5"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C43" s="12" t="s">
+      <c r="C43" s="9" t="s">
         <v>118</v>
       </c>
       <c r="D43" s="5"/>
-      <c r="E43" s="8"/>
+      <c r="E43" s="14"/>
       <c r="F43" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G43" s="5"/>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C44" s="12" t="s">
+      <c r="C44" s="9" t="s">
         <v>119</v>
       </c>
       <c r="D44" s="5"/>
-      <c r="E44" s="8"/>
+      <c r="E44" s="14"/>
       <c r="F44" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G44" s="5"/>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C45" s="12" t="s">
+      <c r="C45" s="9" t="s">
         <v>120</v>
       </c>
       <c r="D45" s="5"/>
-      <c r="E45" s="9"/>
+      <c r="E45" s="15"/>
       <c r="F45" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G45" s="5"/>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="9" t="s">
         <v>80</v>
       </c>
       <c r="C46" t="s">
         <v>123</v>
       </c>
       <c r="D46" s="5"/>
-      <c r="E46" s="7" t="s">
+      <c r="E46" s="13" t="s">
         <v>121</v>
       </c>
       <c r="F46" s="5" t="s">
@@ -1570,56 +1582,56 @@
       <c r="G46" s="5"/>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B47" s="12" t="s">
+      <c r="B47" s="9" t="s">
         <v>81</v>
       </c>
       <c r="C47" t="s">
         <v>124</v>
       </c>
       <c r="D47" s="5"/>
-      <c r="E47" s="8"/>
+      <c r="E47" s="14"/>
       <c r="F47" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G47" s="5"/>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B48" s="12" t="s">
+      <c r="B48" s="9" t="s">
         <v>82</v>
       </c>
       <c r="C48" t="s">
         <v>125</v>
       </c>
       <c r="D48" s="5"/>
-      <c r="E48" s="8"/>
+      <c r="E48" s="14"/>
       <c r="F48" s="5" t="s">
         <v>91</v>
       </c>
       <c r="G48" s="5"/>
     </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B49" s="16" t="s">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B49" s="10" t="s">
         <v>83</v>
       </c>
       <c r="C49" t="s">
         <v>126</v>
       </c>
-      <c r="D49" s="17"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="17" t="s">
+      <c r="D49" s="11"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="G49" s="17"/>
-    </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B50" s="12" t="s">
+      <c r="G49" s="11"/>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B50" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C50" s="12" t="s">
+      <c r="C50" s="9" t="s">
         <v>128</v>
       </c>
       <c r="D50" s="5"/>
-      <c r="E50" s="21" t="s">
+      <c r="E50" s="16" t="s">
         <v>127</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -1627,277 +1639,229 @@
       </c>
       <c r="G50" s="5"/>
     </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B51" s="12" t="s">
+    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B51" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C51" s="12" t="s">
+      <c r="C51" s="9" t="s">
         <v>129</v>
       </c>
       <c r="D51" s="5"/>
-      <c r="E51" s="21"/>
+      <c r="E51" s="16"/>
       <c r="F51" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G51" s="5"/>
     </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B52" s="12" t="s">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B52" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="C52" s="12" t="s">
+      <c r="C52" s="9" t="s">
         <v>130</v>
       </c>
       <c r="D52" s="5"/>
-      <c r="E52" s="21"/>
+      <c r="E52" s="16"/>
       <c r="F52" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G52" s="5"/>
     </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B53" s="12" t="s">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B53" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C53" s="12" t="s">
+      <c r="C53" s="9" t="s">
         <v>131</v>
       </c>
       <c r="D53" s="5"/>
-      <c r="E53" s="21"/>
+      <c r="E53" s="16"/>
       <c r="F53" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G53" s="5"/>
     </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B54" s="18"/>
-      <c r="C54" s="19"/>
-      <c r="D54" s="19"/>
-      <c r="E54" s="19"/>
-      <c r="F54" s="19"/>
-      <c r="G54" s="19"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="20"/>
-    </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B55" s="18"/>
-      <c r="C55" s="19"/>
-      <c r="D55" s="19"/>
-      <c r="E55" s="19"/>
-      <c r="F55" s="19"/>
-      <c r="G55" s="19"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
-    </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B56" s="18"/>
-      <c r="C56" s="19"/>
-      <c r="D56" s="19"/>
-      <c r="E56" s="19"/>
-      <c r="F56" s="19"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="20"/>
-      <c r="I56" s="20"/>
-    </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B57" s="18"/>
-      <c r="C57" s="19"/>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="19"/>
-      <c r="G57" s="19"/>
-      <c r="H57" s="20"/>
-      <c r="I57" s="20"/>
-    </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B58" s="18"/>
-      <c r="C58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="20"/>
-      <c r="I58" s="20"/>
-    </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B59" s="18"/>
-      <c r="C59" s="19"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="20"/>
-      <c r="I59" s="20"/>
-    </row>
-    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B60" s="18"/>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="20"/>
-      <c r="I60" s="20"/>
-    </row>
-    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B61" s="18"/>
-      <c r="C61" s="19"/>
-      <c r="D61" s="19"/>
-      <c r="E61" s="19"/>
-      <c r="F61" s="19"/>
-      <c r="G61" s="19"/>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-    </row>
-    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B62" s="18"/>
-      <c r="C62" s="19"/>
-      <c r="D62" s="19"/>
-      <c r="E62" s="19"/>
-      <c r="F62" s="19"/>
-      <c r="G62" s="19"/>
-      <c r="H62" s="20"/>
-      <c r="I62" s="20"/>
-    </row>
-    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B63" s="18"/>
-      <c r="C63" s="19"/>
-      <c r="D63" s="19"/>
-      <c r="E63" s="19"/>
-      <c r="F63" s="19"/>
-      <c r="G63" s="19"/>
-      <c r="H63" s="20"/>
-      <c r="I63" s="20"/>
-    </row>
-    <row r="64" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B64" s="18"/>
-      <c r="C64" s="19"/>
-      <c r="D64" s="19"/>
-      <c r="E64" s="19"/>
-      <c r="F64" s="19"/>
-      <c r="G64" s="19"/>
-      <c r="H64" s="20"/>
-      <c r="I64" s="20"/>
-    </row>
-    <row r="65" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B65" s="18"/>
-      <c r="C65" s="19"/>
-      <c r="D65" s="19"/>
-      <c r="E65" s="19"/>
-      <c r="F65" s="19"/>
-      <c r="G65" s="19"/>
-      <c r="H65" s="20"/>
-      <c r="I65" s="20"/>
-    </row>
-    <row r="66" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B66" s="18"/>
-      <c r="C66" s="19"/>
-      <c r="D66" s="19"/>
-      <c r="E66" s="19"/>
-      <c r="F66" s="19"/>
-      <c r="G66" s="19"/>
-      <c r="H66" s="20"/>
-      <c r="I66" s="20"/>
-    </row>
-    <row r="67" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B67" s="18"/>
-      <c r="C67" s="19"/>
-      <c r="D67" s="19"/>
-      <c r="E67" s="19"/>
-      <c r="F67" s="19"/>
-      <c r="G67" s="19"/>
-      <c r="H67" s="20"/>
-      <c r="I67" s="20"/>
-    </row>
-    <row r="68" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B68" s="18"/>
-      <c r="C68" s="19"/>
-      <c r="D68" s="19"/>
-      <c r="E68" s="19"/>
-      <c r="F68" s="19"/>
-      <c r="G68" s="19"/>
-      <c r="H68" s="20"/>
-      <c r="I68" s="20"/>
-    </row>
-    <row r="69" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B69" s="18"/>
-      <c r="C69" s="19"/>
-      <c r="D69" s="19"/>
-      <c r="E69" s="19"/>
-      <c r="F69" s="19"/>
-      <c r="G69" s="19"/>
-      <c r="H69" s="20"/>
-      <c r="I69" s="20"/>
-    </row>
-    <row r="70" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B70" s="18"/>
-      <c r="C70" s="19"/>
-      <c r="D70" s="19"/>
-      <c r="E70" s="19"/>
-      <c r="F70" s="19"/>
-      <c r="G70" s="19"/>
-      <c r="H70" s="20"/>
-      <c r="I70" s="20"/>
-    </row>
-    <row r="71" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B71" s="18"/>
-      <c r="C71" s="19"/>
-      <c r="D71" s="19"/>
-      <c r="E71" s="19"/>
-      <c r="F71" s="19"/>
-      <c r="G71" s="19"/>
-      <c r="H71" s="20"/>
-      <c r="I71" s="20"/>
-    </row>
-    <row r="72" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B72" s="18"/>
-      <c r="C72" s="19"/>
-      <c r="D72" s="19"/>
-      <c r="E72" s="19"/>
-      <c r="F72" s="19"/>
-      <c r="G72" s="19"/>
-      <c r="H72" s="20"/>
-      <c r="I72" s="20"/>
-    </row>
-    <row r="73" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B73" s="18"/>
-      <c r="C73" s="19"/>
-      <c r="D73" s="19"/>
-      <c r="E73" s="19"/>
-      <c r="F73" s="19"/>
-      <c r="G73" s="19"/>
-      <c r="H73" s="20"/>
-      <c r="I73" s="20"/>
-    </row>
-    <row r="74" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B74" s="18"/>
-      <c r="C74" s="19"/>
-      <c r="D74" s="19"/>
-      <c r="E74" s="19"/>
-      <c r="F74" s="19"/>
-      <c r="G74" s="19"/>
-      <c r="H74" s="20"/>
-      <c r="I74" s="20"/>
-    </row>
-    <row r="75" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B75" s="20"/>
-      <c r="C75" s="19"/>
-      <c r="D75" s="19"/>
-      <c r="E75" s="19"/>
-      <c r="F75" s="19"/>
-      <c r="G75" s="19"/>
-      <c r="H75" s="20"/>
-      <c r="I75" s="20"/>
-    </row>
-    <row r="76" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B76" s="20"/>
-      <c r="C76" s="19"/>
-      <c r="D76" s="19"/>
-      <c r="E76" s="19"/>
-      <c r="F76" s="19"/>
-      <c r="G76" s="19"/>
-      <c r="H76" s="20"/>
-      <c r="I76" s="20"/>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B54"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="12"/>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B55"/>
+      <c r="C55" s="12"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="12"/>
+      <c r="F55" s="12"/>
+      <c r="G55" s="12"/>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B56"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="12"/>
+      <c r="E56" s="12"/>
+      <c r="F56" s="12"/>
+      <c r="G56" s="12"/>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B57"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B58"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="12"/>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B59"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="12"/>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B60"/>
+      <c r="C60" s="12"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12"/>
+      <c r="F60" s="12"/>
+      <c r="G60" s="12"/>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B61"/>
+      <c r="C61" s="12"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="12"/>
+      <c r="F61" s="12"/>
+      <c r="G61" s="12"/>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B62"/>
+      <c r="C62" s="12"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="12"/>
+      <c r="F62" s="12"/>
+      <c r="G62" s="12"/>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B63"/>
+      <c r="C63" s="12"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="12"/>
+      <c r="F63" s="12"/>
+      <c r="G63" s="12"/>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B64"/>
+      <c r="C64" s="12"/>
+      <c r="D64" s="12"/>
+      <c r="E64" s="12"/>
+      <c r="F64" s="12"/>
+      <c r="G64" s="12"/>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B65"/>
+      <c r="C65" s="12"/>
+      <c r="D65" s="12"/>
+      <c r="E65" s="12"/>
+      <c r="F65" s="12"/>
+      <c r="G65" s="12"/>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B66"/>
+      <c r="C66" s="12"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12"/>
+      <c r="F66" s="12"/>
+      <c r="G66" s="12"/>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B67"/>
+      <c r="C67" s="12"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="12"/>
+      <c r="F67" s="12"/>
+      <c r="G67" s="12"/>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B68"/>
+      <c r="C68" s="12"/>
+      <c r="D68" s="12"/>
+      <c r="E68" s="12"/>
+      <c r="F68" s="12"/>
+      <c r="G68" s="12"/>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B69"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="12"/>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="12"/>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B70"/>
+      <c r="C70" s="12"/>
+      <c r="D70" s="12"/>
+      <c r="E70" s="12"/>
+      <c r="F70" s="12"/>
+      <c r="G70" s="12"/>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B71"/>
+      <c r="C71" s="12"/>
+      <c r="D71" s="12"/>
+      <c r="E71" s="12"/>
+      <c r="F71" s="12"/>
+      <c r="G71" s="12"/>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B72"/>
+      <c r="C72" s="12"/>
+      <c r="D72" s="12"/>
+      <c r="E72" s="12"/>
+      <c r="F72" s="12"/>
+      <c r="G72" s="12"/>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B73"/>
+      <c r="C73" s="12"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12"/>
+      <c r="F73" s="12"/>
+      <c r="G73" s="12"/>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B74"/>
+      <c r="C74" s="12"/>
+      <c r="D74" s="12"/>
+      <c r="E74" s="12"/>
+      <c r="F74" s="12"/>
+      <c r="G74" s="12"/>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="C75" s="12"/>
+      <c r="D75" s="12"/>
+      <c r="E75" s="12"/>
+      <c r="F75" s="12"/>
+      <c r="G75" s="12"/>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="C76" s="12"/>
+      <c r="D76" s="12"/>
+      <c r="E76" s="12"/>
+      <c r="F76" s="12"/>
+      <c r="G76" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
bugfix: correct CI frontend
</commit_message>
<xml_diff>
--- a/docs/Producto_Backlog_V1.0.xlsx
+++ b/docs/Producto_Backlog_V1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jhoan\Documents\Programacion\posSYSTEM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39E53EF1-BA16-4ACC-9414-6F460BDAECF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E1133D1-B6A7-4878-A733-4FC0A9C116D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="134">
   <si>
     <t>Columna</t>
   </si>
@@ -1212,7 +1212,9 @@
       <c r="C21" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="D21" s="5"/>
+      <c r="D21" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="E21" s="13" t="s">
         <v>92</v>
       </c>
@@ -1228,7 +1230,9 @@
       <c r="C22" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="D22" s="5"/>
+      <c r="D22" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="E22" s="14"/>
       <c r="F22" s="5" t="s">
         <v>49</v>
@@ -1242,7 +1246,9 @@
       <c r="C23" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D23" s="5"/>
+      <c r="D23" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="E23" s="14"/>
       <c r="F23" s="5" t="s">
         <v>49</v>
@@ -1256,7 +1262,9 @@
       <c r="C24" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D24" s="5"/>
+      <c r="D24" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="E24" s="15"/>
       <c r="F24" s="5" t="s">
         <v>91</v>
@@ -1328,7 +1336,9 @@
       <c r="C29" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="D29" s="5"/>
+      <c r="D29" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="E29" s="17" t="s">
         <v>107</v>
       </c>
@@ -1344,7 +1354,9 @@
       <c r="C30" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="D30" s="5"/>
+      <c r="D30" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="E30" s="18"/>
       <c r="F30" s="5" t="s">
         <v>23</v>
@@ -1358,7 +1370,9 @@
       <c r="C31" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="D31" s="5"/>
+      <c r="D31" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="E31" s="18"/>
       <c r="F31" s="5" t="s">
         <v>23</v>
@@ -1372,7 +1386,9 @@
       <c r="C32" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="D32" s="5"/>
+      <c r="D32" s="5" t="s">
+        <v>133</v>
+      </c>
       <c r="E32" s="18"/>
       <c r="F32" s="5" t="s">
         <v>49</v>

</xml_diff>